<commit_message>
chore: align SurgeBlade workbook column with thrust width
Keep the balancing sheet export on width 0.8 instead of the old slash angle.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Tools/BalancingSheets/output/NeoSurvive_Balancing.xlsx
+++ b/Tools/BalancingSheets/output/NeoSurvive_Balancing.xlsx
@@ -2385,7 +2385,7 @@
       </c>
       <c r="E1" s="8" t="inlineStr">
         <is>
-          <t>angle</t>
+          <t>width</t>
         </is>
       </c>
       <c r="F1" s="8" t="inlineStr">
@@ -2430,7 +2430,7 @@
         <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="F2" t="n">
         <v>1.2</v>
@@ -2464,7 +2464,7 @@
         <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="F3" t="n">
         <v>1.2</v>
@@ -2498,7 +2498,7 @@
         <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="F4" t="n">
         <v>1.2</v>
@@ -2532,7 +2532,7 @@
         <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="F5" t="n">
         <v>1.2</v>
@@ -2566,7 +2566,7 @@
         <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="F6" t="n">
         <v>1.2</v>

</xml_diff>